<commit_message>
Recalculated all models that aren't oversized
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows_code\Statistical_Analysis_Lambda_Catalog\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LocalPython\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D477202-9FFB-4C3D-B175-167A56CC28CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{344494EC-7ED4-4477-B268-9C614ECDA867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression Instructions" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="176">
   <si>
     <t>To analyze your own dataset, copy the Regression sheet into your workbook (right-click the tab → Move or Copy). This carries over all workbook-scoped LAMBDA functions as well as the sheet-scoped names the Regression sheet uses.</t>
   </si>
@@ -573,6 +573,36 @@
   </si>
   <si>
     <t>The analysis sample is derived automatically — a row is included when the Response is numeric, every included Continuous predictor is numeric, and every Filter column is truthy. Include settings and Log (drop ≤ 0) also affect the sample. Categorical predictors impose no completeness requirement: rows with a blank category still enter the sample (all of that variable's dummies are blank there) unless a Filter excludes them.</t>
+  </si>
+  <si>
+    <t>RESIDUALS UNDER FIXED EFFECTS</t>
+  </si>
+  <si>
+    <t>What you'll see</t>
+  </si>
+  <si>
+    <t>What it means</t>
+  </si>
+  <si>
+    <t>How to read it</t>
+  </si>
+  <si>
+    <t>The response-scale Residual Output headers relabel: Predicted Y, Residuals, and PRESS Residual gain "(Within &lt;FE variable&gt;)" and Y becomes "Deviation from &lt;FE variable&gt; Avg."</t>
+  </si>
+  <si>
+    <t>Once a Fixed Effects row is declared, every diagnostic column is computed from the within (group-demeaned) fit. The model absorbs a separate intercept per group, so each column holds deviations from the group's own average, not from the pooled response. The dimensionless columns (Hat Diagonal, Studentized Residuals, Cook's Distance, Scale-Location, …) keep their names — they were never in response units.</t>
+  </si>
+  <si>
+    <t>The Tier 1 and Tier 2 plots read these same within-group values: a funnel means non-constant variance within groups, a curve means the within-group relationship is misspecified. Between-group differences no longer appear in the residuals at all — absorbing them is the point of Fixed Effects.</t>
+  </si>
+  <si>
+    <t>Each group's Deviation values average zero by construction; Durbin-Watson reads "n/a — FE active" and the BFN Panel Durbin-Watson row below it takes over.</t>
+  </si>
+  <si>
+    <t>The demeaning centers every group on zero, so a large Deviation is a row far from its own group's average — the quantity the model actually fits. Classical Durbin-Watson assumes one ordered series; with a Sequence axis and Fixed Effects the residuals form panels, so serial correlation is read with the Bhargava–Franzini–Narendranathan (1982) panel statistic instead.</t>
+  </si>
+  <si>
+    <t>Treat the BFN cell as the DW cell's replacement while Fixed Effects is active — the classical DW bounds do not apply to panel residuals. The influence flags (Cook's Distance, PRESS) apply unchanged, now measuring influence on the within-group fit.</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1687EF57-B6EB-444E-A46B-98E7D5CA1EC6}">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1484,6 +1514,46 @@
       </c>
       <c r="C38" s="2" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="300" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="270" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand modeling filter guidance
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -1389,95 +1389,95 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="165" customHeight="1">
+    <row r="5" ht="225" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sample Filtering &amp; Completeness
+(Role = Filter)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Add TRUE/FALSE filter columns to the source dataset to define the population for a model without deleting or rearranging observations. Keeping alternative filters as separate columns makes it quick to fit related model specifications and to test how sensitive the results are to removing individual observations.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>The active Filter columns are combined with AND: a row is included only when every Filter is TRUE. The Response and every included Continuous predictor must also be numeric (listwise deletion). Categorical predictors impose no completeness condition — a blank category is simply not a level. Log (drop ≤ 0) adds its own exclusion layer, and excluded-row counts surface in the status cells above the spec (B2 / G2).</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Add one filter for the target population and additional candidate filters for common subsets. Switch each column's Role between Filter and Exclude to generate related models quickly. For point-removal sensitivity analysis, add a column that is TRUE for every row except the observation being tested; activating it refits the model without that point while leaving the source data intact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="165" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Intercept Control
 (C2 toggle)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>The intercept is the model's baseline — the expected response at zero on every predictor. Keep the intercept unless the model requires a zero response when all predictors are zero; the baseline need not itself be a meaningful observed case.</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>A model-level on/off toggle (cell C2). With reference-coded categoricals in the model, turning it OFF is flagged red: the workbook still drops the reference category, so removing the intercept also constrains the reference baseline to zero. Under Fixed Effects it is flagged because the within transformation demeans the data, and the intercept of demeaned data is an uninterpretable artifact.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Theory says cost is zero at zero production, or the instrument reads zero with no input? Turn the intercept off for a regression-through-origin fit. Otherwise leave it on and let it absorb the reference levels' baseline.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="165" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7" ht="165" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Reference Levels
 (Categorical predictors)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>A categorical column cannot enter a regression as text — it has to become numbers. But one 0/1 column per level PLUS an intercept is redundant (perfect multicollinearity), so one level must step aside as the baseline everything else is measured against.</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Treatment (dummy) coding: a 0/1 column per retained level, with the reference level dropped. Each categorical coefficient reads as a contrast against the reference; the intercept absorbs the reference level's baseline. The default reference is the first-in-sort-order level; type another in column E to override. A typed level not present in the sample is flagged red, never silently fitted.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Origin (US / Europe / Japan) predicting MPG: with US as the reference, the Europe coefficient is the Europe-vs-US difference in MPG. Pick the level that makes the contrasts meaningful — an experiment's control group, or the market standard your question is 'compared to what?'</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="345" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="345" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Log Transforms
 (Transform = Log / Log (drop ≤ 0))</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Log transforms can represent multiplicative relationships. They change the scale on which the model is fitted and its coefficients are interpreted; they do not guarantee an adequate fit or symmetric residuals.</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Only variables marked Log are transformed. Logging a predictor alone leaves the response and residuals in response units. When the response is logged, Naive exponentiates its fitted log value; Duan also multiplies by the average of exp(residuals). This common smearing factor estimates an original-unit conditional mean only when the error retransformation factor is constant across predictor values. It does not generally correct heteroscedasticity. Naive represents a conditional median when log errors have conditional median zero. Original-unit interval bounds always use Naive; they are not confidence bounds for the Duan-adjusted mean. Zeros and negatives have no logarithm: plain Log keeps them in the sample and the fit returns #N/A and flags the Transform cell red; Log (drop ≤ 0) excludes them and reports how many.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>In a log-log model without interactions, a coefficient gives the proportional change in the fitted geometric mean of the response for a proportional change in that predictor, holding other predictors fixed. For small changes, a 1% predictor increase corresponds to approximately that coefficient percent change in the fitted response. Inspect residual plots after transformation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="180" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Sample Filtering &amp; Completeness
-(Role = Filter)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>The fit should answer a question about a specific population, and rows with missing values cannot be part of it. The workbook derives the analysis sample from the spec, so a change of population is a specification change — not hand-deleting rows on the data sheet.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>A per-row mask ANDed together: every Filter column must be TRUE, the Response must be numeric, and every included Continuous predictor must be numeric (listwise deletion). Categorical predictors impose no completeness condition — a blank category is just not a level. Log (drop ≤ 0) adds its own exclusion layer, and the excluded-row counts surface in the status cells above the spec (B2 / G2) rather than staying silent.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Restrict a nationwide demand model to one market segment: add a derived column that is TRUE only for that segment, set its Role to Filter, and every statistic is refit to that population. Retarget the filter later and the sample follows — the data sheet is never touched.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: how to add models and rows on the Model Comparison sheet
Adds a "Using the Model Comparison sheet" section to the Model Comparison
Guide: copy a model sheet with Move or Copy (never paste its cells, which
leaves formulas reading the original sheet's sheet-scoped names), point a
spare Comp_Anchor_<n> row at it, add a new anchor name plus row when the
spares run out, and choose the reference row.

The new constant is pinned in the freshness test. The template was patched
at the XML level on a machine without Excel; re-run
scripts/rebuild_static_sheets.py on the Excel machine to replace it with a
true regeneration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019sY6pBYvJv1bHKVSmALV7c
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="425">
   <si>
     <t>MODELING CONCEPTS — THE WHY BEHIND EACH FEATURE</t>
   </si>
@@ -1272,6 +1272,66 @@
   </si>
   <si>
     <t>Fitting a model is the easy half. The hard half is deciding which of several specifications to report, on what evidence, and whether lining them up is legitimate at all. This sheet answers that in four layers: the conditions that make two models comparable, what each statistic is for and what change it survives, a step-by-step procedure for choosing a specification, and the moves that look like comparisons and are not. It is a reading guide only — it adds no formulas and no new named ranges. The Model Comparison sheet beside it is the registry this guide explains: one row per fitted model, with the comparability tests the first layer below describes already applied to each row. For the mechanics of setting a specification up, see the Regression Instructions sheet; for what each modeling feature does, see Modeling Concepts; for what to look for in the residual plots, see the Diagnostic Guide.</t>
+  </si>
+  <si>
+    <t>USING THE MODEL COMPARISON SHEET — ADDING MODELS AND ROWS</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Where</t>
+  </si>
+  <si>
+    <t>Why it matters</t>
+  </si>
+  <si>
+    <t>Create another model — copy the whole sheet</t>
+  </si>
+  <si>
+    <t>Right-click the sheet tab of the Regression template sheet, or of any model sheet already fitted, then choose Move or Copy… and tick Create a copy.</t>
+  </si>
+  <si>
+    <t>Rename the copy, then edit its Model Specification. A sheet copied this way arrives with its own set of sheet-scoped names — the spec wiring, the constructor closures, the chart ranges and the Comparison_Anchor the registry reads — every one scoped to the new sheet, so the copy fits its own specification and nothing else.</t>
+  </si>
+  <si>
+    <t>Never select the cells and copy, or cut, and paste them onto a blank sheet. The formulas come across but the sheet-scoped names do not, so every formula keeps reading the ORIGINAL sheet: the new sheet shows the old model's numbers. Nothing errors — it is a silent wrong answer.</t>
+  </si>
+  <si>
+    <t>Point a spare row at the new model</t>
+  </si>
+  <si>
+    <t>Formulas &gt; Name Manager, with the Model Comparison sheet active. The Anchor column on that sheet shows the address each row reads.</t>
+  </si>
+  <si>
+    <t>Every row owns a sheet-scoped name, Comp_Anchor_1, Comp_Anchor_2 and so on, numbered from the first data row (row 4 is Comp_Anchor_1). The build ships three spare rows whose anchors point at the sheet's own $A$1. Edit the first spare one so Refers To reads ='&lt;new sheet&gt;'!$AF$3 — the model sheet's response-label cell — and every cell in the row fills in.</t>
+  </si>
+  <si>
+    <t>A spare row reads blank until it is pointed at a model sheet, and a mis-pointed row stays blank rather than reading an unrelated cell: the readers check for the MODEL SPECIFICATION heading at the target's A1 before reading anything.</t>
+  </si>
+  <si>
+    <t>Add a row when the spare rows run out</t>
+  </si>
+  <si>
+    <t>Name Manager first, then the first empty row directly below the table.</t>
+  </si>
+  <si>
+    <t>1. Name Manager &gt; New: Name Comp_Anchor_&lt;n+1&gt;, the next unused number; Scope Model Comparison, not Workbook; Refers To ='&lt;model sheet&gt;'!$AF$3. 2. Select the table's last row across every column and copy it down one row. 3. With only the new row selected, Find &amp; Replace Comp_Anchor_&lt;n&gt; with Comp_Anchor_&lt;n+1&gt;, looking in Formulas.</t>
+  </si>
+  <si>
+    <t>A copied row still reads the name the row above it reads, so skipping step 3 duplicates the previous model instead of adding one. Replace within the new row only. The gate flags, the row-2 verdicts and the zone shading already reach row 103, so a new row down to there is counted with no other edit.</t>
+  </si>
+  <si>
+    <t>Choose the reference model</t>
+  </si>
+  <si>
+    <t>The first data row, row 4 — the name Comp_Anchor_1.</t>
+  </si>
+  <si>
+    <t>Every gate column (Same Set?, Same Space?, Same Method?, Same Inputs?) compares its row against this one. To compare the others against a different model, point Comp_Anchor_1 at that model's sheet.</t>
+  </si>
+  <si>
+    <t>The row-2 verdicts count how many rows agree with the reference, so a reference that is itself the odd one out shades every other row. Pick the specification the rest are variations on.</t>
   </si>
 </sst>
 </file>
@@ -2479,7 +2539,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A060BA2-BEC8-4428-B2E8-8EF51D7CB23B}">
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -3332,41 +3392,119 @@
         <v>376</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="5"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="B86" s="5"/>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="4" t="s">
+      <c r="B93" s="5"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
         <v>378</v>
       </c>
-      <c r="B87" s="4" t="s">
+      <c r="B94" s="4" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A88" s="2" t="s">
+    <row r="95" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B95" s="2" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
+    <row r="96" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B96" s="2" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
+    <row r="97" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B97" s="2" t="s">
         <v>385</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the dist with the new sheet
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows_code\Statistical_Analysis_Lambda_Catalog\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\local_python\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E33E69BA-68A3-4EED-8A1D-9A2190B1BC55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEAFADBF-4B53-4D21-A8C1-06020F14674A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression Instructions" sheetId="1" r:id="rId1"/>
@@ -3348,7 +3348,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>365</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>368</v>
       </c>
@@ -3370,7 +3370,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>371</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>374</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>409</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" ht="120" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>413</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" ht="120" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>417</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>421</v>
       </c>
@@ -3470,13 +3470,13 @@
         <v>424</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>377</v>
       </c>
       <c r="B93" s="5"/>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>378</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>380</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>382</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>384</v>
       </c>

</xml_diff>